<commit_message>
Fixed error in dataset
</commit_message>
<xml_diff>
--- a/plga_dataset/mp_dataset_initial_formulation.xlsx
+++ b/plga_dataset/mp_dataset_initial_formulation.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sanan\Desktop\phd\paper1\A Dataset on Formulation Parameters and Characteristics of Drug-Loaded PLGA Microparticles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sanan\Downloads\data_check\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{562B9B29-D786-4104-9545-C1F923A7BB6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{795F45B4-E5DB-4F07-BCA0-B7417333DF21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$Q$322</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$O$322</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1336" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1299" uniqueCount="309">
   <si>
     <t>Formulation Index</t>
   </si>
@@ -950,39 +950,6 @@
   </si>
   <si>
     <t>olanzapine</t>
-  </si>
-  <si>
-    <t>release_profile_shape</t>
-  </si>
-  <si>
-    <t>note</t>
-  </si>
-  <si>
-    <t>between 1 and 2</t>
-  </si>
-  <si>
-    <t>looks like 4, but no burst actually</t>
-  </si>
-  <si>
-    <t>?</t>
-  </si>
-  <si>
-    <t>bad sampling</t>
-  </si>
-  <si>
-    <t>wtf</t>
-  </si>
-  <si>
-    <t>no really burst</t>
-  </si>
-  <si>
-    <t>no really latent</t>
-  </si>
-  <si>
-    <t>or 2</t>
-  </si>
-  <si>
-    <t>close to 4</t>
   </si>
 </sst>
 </file>
@@ -1011,7 +978,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1034,27 +1001,13 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -1359,7 +1312,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q322"/>
+  <dimension ref="A1:O322"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.44140625" bestFit="1" customWidth="1"/>
@@ -1377,10 +1330,9 @@
     <col min="13" max="13" width="26.21875" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="30.109375" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="34" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="19.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1426,14 +1378,8 @@
       <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="2" t="s">
-        <v>309</v>
-      </c>
-      <c r="Q1" s="2" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1470,11 +1416,8 @@
       <c r="O2" t="s">
         <v>18</v>
       </c>
-      <c r="P2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1511,11 +1454,8 @@
       <c r="O3" t="s">
         <v>22</v>
       </c>
-      <c r="P3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1552,14 +1492,8 @@
       <c r="O4" t="s">
         <v>22</v>
       </c>
-      <c r="P4">
-        <v>1</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1596,14 +1530,8 @@
       <c r="O5" t="s">
         <v>22</v>
       </c>
-      <c r="P5">
-        <v>1</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1640,14 +1568,8 @@
       <c r="O6" t="s">
         <v>22</v>
       </c>
-      <c r="P6">
-        <v>1</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1684,11 +1606,8 @@
       <c r="O7" t="s">
         <v>22</v>
       </c>
-      <c r="P7">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1725,14 +1644,8 @@
       <c r="O8" t="s">
         <v>22</v>
       </c>
-      <c r="P8">
-        <v>1</v>
-      </c>
-      <c r="Q8" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1769,11 +1682,8 @@
       <c r="O9" t="s">
         <v>22</v>
       </c>
-      <c r="P9">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1810,11 +1720,8 @@
       <c r="O10" t="s">
         <v>22</v>
       </c>
-      <c r="P10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1851,11 +1758,8 @@
       <c r="O11" t="s">
         <v>22</v>
       </c>
-      <c r="P11">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1892,11 +1796,8 @@
       <c r="O12" t="s">
         <v>22</v>
       </c>
-      <c r="P12">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1933,11 +1834,8 @@
       <c r="O13" t="s">
         <v>22</v>
       </c>
-      <c r="P13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1974,11 +1872,8 @@
       <c r="O14" t="s">
         <v>22</v>
       </c>
-      <c r="P14">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -2015,11 +1910,8 @@
       <c r="O15" t="s">
         <v>22</v>
       </c>
-      <c r="P15">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -2056,11 +1948,8 @@
       <c r="O16" t="s">
         <v>22</v>
       </c>
-      <c r="P16">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -2097,11 +1986,8 @@
       <c r="O17" t="s">
         <v>22</v>
       </c>
-      <c r="P17">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -2138,11 +2024,8 @@
       <c r="O18" t="s">
         <v>22</v>
       </c>
-      <c r="P18">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -2179,11 +2062,8 @@
       <c r="O19" t="s">
         <v>22</v>
       </c>
-      <c r="P19">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -2220,11 +2100,8 @@
       <c r="O20" t="s">
         <v>22</v>
       </c>
-      <c r="P20">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -2261,11 +2138,8 @@
       <c r="O21" t="s">
         <v>22</v>
       </c>
-      <c r="P21">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -2302,11 +2176,8 @@
       <c r="O22" t="s">
         <v>27</v>
       </c>
-      <c r="P22">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -2343,14 +2214,8 @@
       <c r="O23" t="s">
         <v>27</v>
       </c>
-      <c r="P23">
-        <v>3</v>
-      </c>
-      <c r="Q23" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -2387,14 +2252,8 @@
       <c r="O24" t="s">
         <v>27</v>
       </c>
-      <c r="P24">
-        <v>3</v>
-      </c>
-      <c r="Q24" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
@@ -2431,14 +2290,8 @@
       <c r="O25" t="s">
         <v>27</v>
       </c>
-      <c r="P25">
-        <v>3</v>
-      </c>
-      <c r="Q25" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -2475,14 +2328,8 @@
       <c r="O26" t="s">
         <v>27</v>
       </c>
-      <c r="P26">
-        <v>3</v>
-      </c>
-      <c r="Q26" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
@@ -2519,11 +2366,8 @@
       <c r="O27" t="s">
         <v>30</v>
       </c>
-      <c r="P27">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>27</v>
       </c>
@@ -2560,14 +2404,8 @@
       <c r="O28" t="s">
         <v>33</v>
       </c>
-      <c r="P28">
-        <v>3</v>
-      </c>
-      <c r="Q28" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
@@ -2604,14 +2442,8 @@
       <c r="O29" t="s">
         <v>33</v>
       </c>
-      <c r="P29">
-        <v>3</v>
-      </c>
-      <c r="Q29" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
@@ -2648,11 +2480,8 @@
       <c r="O30" t="s">
         <v>33</v>
       </c>
-      <c r="P30">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
@@ -2689,11 +2518,8 @@
       <c r="O31" t="s">
         <v>37</v>
       </c>
-      <c r="P31">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>31</v>
       </c>
@@ -2730,11 +2556,8 @@
       <c r="O32" t="s">
         <v>37</v>
       </c>
-      <c r="P32">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>32</v>
       </c>
@@ -2771,11 +2594,8 @@
       <c r="O33" t="s">
         <v>40</v>
       </c>
-      <c r="P33">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>33</v>
       </c>
@@ -2812,11 +2632,8 @@
       <c r="O34" t="s">
         <v>40</v>
       </c>
-      <c r="P34">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>34</v>
       </c>
@@ -2853,11 +2670,8 @@
       <c r="O35" t="s">
         <v>40</v>
       </c>
-      <c r="P35">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>35</v>
       </c>
@@ -2894,11 +2708,8 @@
       <c r="O36" t="s">
         <v>43</v>
       </c>
-      <c r="P36">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>36</v>
       </c>
@@ -2935,11 +2746,8 @@
       <c r="O37" t="s">
         <v>43</v>
       </c>
-      <c r="P37">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>37</v>
       </c>
@@ -2976,11 +2784,8 @@
       <c r="O38" t="s">
         <v>46</v>
       </c>
-      <c r="P38">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>38</v>
       </c>
@@ -3017,11 +2822,8 @@
       <c r="O39" t="s">
         <v>46</v>
       </c>
-      <c r="P39">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>39</v>
       </c>
@@ -3058,11 +2860,8 @@
       <c r="O40" t="s">
         <v>49</v>
       </c>
-      <c r="P40">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>40</v>
       </c>
@@ -3099,11 +2898,8 @@
       <c r="O41" t="s">
         <v>52</v>
       </c>
-      <c r="P41">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>41</v>
       </c>
@@ -3140,11 +2936,8 @@
       <c r="O42" t="s">
         <v>52</v>
       </c>
-      <c r="P42">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>42</v>
       </c>
@@ -3181,14 +2974,8 @@
       <c r="O43" t="s">
         <v>52</v>
       </c>
-      <c r="P43">
-        <v>4</v>
-      </c>
-      <c r="Q43" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="44" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>43</v>
       </c>
@@ -3225,14 +3012,8 @@
       <c r="O44" t="s">
         <v>58</v>
       </c>
-      <c r="P44">
-        <v>4</v>
-      </c>
-      <c r="Q44" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="45" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>44</v>
       </c>
@@ -3269,11 +3050,8 @@
       <c r="O45" t="s">
         <v>58</v>
       </c>
-      <c r="P45">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="46" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>45</v>
       </c>
@@ -3310,11 +3088,8 @@
       <c r="O46" t="s">
         <v>61</v>
       </c>
-      <c r="P46">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="47" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="47" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>46</v>
       </c>
@@ -3351,11 +3126,8 @@
       <c r="O47" t="s">
         <v>64</v>
       </c>
-      <c r="P47">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="48" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="48" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>47</v>
       </c>
@@ -3392,11 +3164,8 @@
       <c r="O48" t="s">
         <v>67</v>
       </c>
-      <c r="P48">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="49" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>48</v>
       </c>
@@ -3433,11 +3202,8 @@
       <c r="O49" t="s">
         <v>70</v>
       </c>
-      <c r="P49">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="50" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>49</v>
       </c>
@@ -3474,11 +3240,8 @@
       <c r="O50" t="s">
         <v>70</v>
       </c>
-      <c r="P50">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="51" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>50</v>
       </c>
@@ -3515,11 +3278,8 @@
       <c r="O51" t="s">
         <v>71</v>
       </c>
-      <c r="P51">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="52" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>51</v>
       </c>
@@ -3556,11 +3316,8 @@
       <c r="O52" t="s">
         <v>71</v>
       </c>
-      <c r="P52">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="53" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>52</v>
       </c>
@@ -3597,11 +3354,8 @@
       <c r="O53" t="s">
         <v>71</v>
       </c>
-      <c r="P53">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="54" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>53</v>
       </c>
@@ -3638,11 +3392,8 @@
       <c r="O54" t="s">
         <v>71</v>
       </c>
-      <c r="P54">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="55" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>54</v>
       </c>
@@ -3679,11 +3430,8 @@
       <c r="O55" t="s">
         <v>71</v>
       </c>
-      <c r="P55">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="56" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>55</v>
       </c>
@@ -3720,11 +3468,8 @@
       <c r="O56" t="s">
         <v>71</v>
       </c>
-      <c r="P56">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="57" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>56</v>
       </c>
@@ -3761,11 +3506,8 @@
       <c r="O57" t="s">
         <v>71</v>
       </c>
-      <c r="P57">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="58" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="58" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>57</v>
       </c>
@@ -3802,11 +3544,8 @@
       <c r="O58" t="s">
         <v>84</v>
       </c>
-      <c r="P58">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="59" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="59" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>58</v>
       </c>
@@ -3843,11 +3582,8 @@
       <c r="O59" t="s">
         <v>87</v>
       </c>
-      <c r="P59">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="60" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="60" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>59</v>
       </c>
@@ -3884,11 +3620,8 @@
       <c r="O60" t="s">
         <v>90</v>
       </c>
-      <c r="P60">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="61" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>60</v>
       </c>
@@ -3925,11 +3658,8 @@
       <c r="O61" t="s">
         <v>90</v>
       </c>
-      <c r="P61">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="62" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="62" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>61</v>
       </c>
@@ -3966,11 +3696,8 @@
       <c r="O62" t="s">
         <v>91</v>
       </c>
-      <c r="P62">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="63" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>62</v>
       </c>
@@ -4007,11 +3734,8 @@
       <c r="O63" t="s">
         <v>91</v>
       </c>
-      <c r="P63">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="64" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="64" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>63</v>
       </c>
@@ -4048,11 +3772,8 @@
       <c r="O64" t="s">
         <v>94</v>
       </c>
-      <c r="P64">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="65" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="65" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>64</v>
       </c>
@@ -4089,11 +3810,8 @@
       <c r="O65" t="s">
         <v>97</v>
       </c>
-      <c r="P65">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="66" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="66" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>65</v>
       </c>
@@ -4130,11 +3848,8 @@
       <c r="O66" t="s">
         <v>97</v>
       </c>
-      <c r="P66">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="67" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="67" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>66</v>
       </c>
@@ -4171,11 +3886,8 @@
       <c r="O67" t="s">
         <v>97</v>
       </c>
-      <c r="P67">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="68" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="68" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>67</v>
       </c>
@@ -4212,11 +3924,8 @@
       <c r="O68" t="s">
         <v>100</v>
       </c>
-      <c r="P68">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="69" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="69" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>68</v>
       </c>
@@ -4253,11 +3962,8 @@
       <c r="O69" t="s">
         <v>100</v>
       </c>
-      <c r="P69">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="70" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="70" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>69</v>
       </c>
@@ -4294,11 +4000,8 @@
       <c r="O70" t="s">
         <v>103</v>
       </c>
-      <c r="P70">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="71" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="71" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>70</v>
       </c>
@@ -4335,11 +4038,8 @@
       <c r="O71" t="s">
         <v>103</v>
       </c>
-      <c r="Q71" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="72" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="72" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>71</v>
       </c>
@@ -4376,11 +4076,8 @@
       <c r="O72" t="s">
         <v>103</v>
       </c>
-      <c r="P72">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="73" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="73" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>72</v>
       </c>
@@ -4417,11 +4114,8 @@
       <c r="O73" t="s">
         <v>103</v>
       </c>
-      <c r="P73">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="74" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="74" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>73</v>
       </c>
@@ -4458,14 +4152,8 @@
       <c r="O74" t="s">
         <v>103</v>
       </c>
-      <c r="P74">
-        <v>4</v>
-      </c>
-      <c r="Q74" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="75" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="75" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>74</v>
       </c>
@@ -4502,14 +4190,8 @@
       <c r="O75" t="s">
         <v>103</v>
       </c>
-      <c r="P75">
-        <v>4</v>
-      </c>
-      <c r="Q75" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="76" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="76" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>75</v>
       </c>
@@ -4546,11 +4228,8 @@
       <c r="O76" t="s">
         <v>103</v>
       </c>
-      <c r="P76">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="77" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="77" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>76</v>
       </c>
@@ -4587,11 +4266,8 @@
       <c r="O77" t="s">
         <v>103</v>
       </c>
-      <c r="P77">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="78" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="78" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>77</v>
       </c>
@@ -4628,14 +4304,8 @@
       <c r="O78" t="s">
         <v>103</v>
       </c>
-      <c r="P78">
-        <v>4</v>
-      </c>
-      <c r="Q78" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="79" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="79" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>78</v>
       </c>
@@ -4672,14 +4342,8 @@
       <c r="O79" t="s">
         <v>103</v>
       </c>
-      <c r="P79">
-        <v>4</v>
-      </c>
-      <c r="Q79" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="80" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="80" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>79</v>
       </c>
@@ -4716,14 +4380,8 @@
       <c r="O80" t="s">
         <v>103</v>
       </c>
-      <c r="P80">
-        <v>4</v>
-      </c>
-      <c r="Q80" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="81" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="81" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>80</v>
       </c>
@@ -4760,11 +4418,8 @@
       <c r="O81" t="s">
         <v>103</v>
       </c>
-      <c r="P81">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="82" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="82" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>81</v>
       </c>
@@ -4801,11 +4456,8 @@
       <c r="O82" t="s">
         <v>106</v>
       </c>
-      <c r="P82">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="83" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="83" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>82</v>
       </c>
@@ -4842,11 +4494,8 @@
       <c r="O83" t="s">
         <v>107</v>
       </c>
-      <c r="P83">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="84" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="84" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>83</v>
       </c>
@@ -4883,11 +4532,8 @@
       <c r="O84" t="s">
         <v>107</v>
       </c>
-      <c r="P84">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="85" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="85" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>84</v>
       </c>
@@ -4924,11 +4570,8 @@
       <c r="O85" t="s">
         <v>107</v>
       </c>
-      <c r="P85">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="86" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="86" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>85</v>
       </c>
@@ -4965,14 +4608,8 @@
       <c r="O86" t="s">
         <v>110</v>
       </c>
-      <c r="P86">
-        <v>4</v>
-      </c>
-      <c r="Q86" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="87" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="87" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>86</v>
       </c>
@@ -5009,11 +4646,8 @@
       <c r="O87" t="s">
         <v>110</v>
       </c>
-      <c r="P87">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="88" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="88" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>87</v>
       </c>
@@ -5050,11 +4684,8 @@
       <c r="O88" t="s">
         <v>110</v>
       </c>
-      <c r="P88">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="89" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="89" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>88</v>
       </c>
@@ -5091,11 +4722,8 @@
       <c r="O89" t="s">
         <v>110</v>
       </c>
-      <c r="P89">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="90" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="90" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>89</v>
       </c>
@@ -5132,11 +4760,8 @@
       <c r="O90" t="s">
         <v>112</v>
       </c>
-      <c r="P90">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="91" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="91" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>90</v>
       </c>
@@ -5173,11 +4798,8 @@
       <c r="O91" t="s">
         <v>112</v>
       </c>
-      <c r="P91">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="92" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="92" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>91</v>
       </c>
@@ -5214,11 +4836,8 @@
       <c r="O92" t="s">
         <v>112</v>
       </c>
-      <c r="P92">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="93" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="93" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>92</v>
       </c>
@@ -5255,11 +4874,8 @@
       <c r="O93" t="s">
         <v>112</v>
       </c>
-      <c r="P93">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="94" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="94" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>93</v>
       </c>
@@ -5296,11 +4912,8 @@
       <c r="O94" t="s">
         <v>112</v>
       </c>
-      <c r="P94">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="95" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="95" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>94</v>
       </c>
@@ -5337,11 +4950,8 @@
       <c r="O95" t="s">
         <v>112</v>
       </c>
-      <c r="P95">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="96" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="96" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>95</v>
       </c>
@@ -5378,11 +4988,8 @@
       <c r="O96" t="s">
         <v>112</v>
       </c>
-      <c r="P96">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="97" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="97" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>96</v>
       </c>
@@ -5419,11 +5026,8 @@
       <c r="O97" t="s">
         <v>112</v>
       </c>
-      <c r="P97">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="98" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="98" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>97</v>
       </c>
@@ -5460,11 +5064,8 @@
       <c r="O98" t="s">
         <v>115</v>
       </c>
-      <c r="P98">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="99" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="99" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>98</v>
       </c>
@@ -5501,11 +5102,8 @@
       <c r="O99" t="s">
         <v>115</v>
       </c>
-      <c r="P99">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="100" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="100" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A100">
         <v>99</v>
       </c>
@@ -5542,11 +5140,8 @@
       <c r="O100" t="s">
         <v>115</v>
       </c>
-      <c r="P100">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="101" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="101" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A101">
         <v>100</v>
       </c>
@@ -5583,11 +5178,8 @@
       <c r="O101" t="s">
         <v>118</v>
       </c>
-      <c r="P101">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="102" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="102" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A102">
         <v>101</v>
       </c>
@@ -5624,11 +5216,8 @@
       <c r="O102" t="s">
         <v>118</v>
       </c>
-      <c r="P102">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="103" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="103" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A103">
         <v>102</v>
       </c>
@@ -5665,11 +5254,8 @@
       <c r="O103" t="s">
         <v>118</v>
       </c>
-      <c r="P103">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="104" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="104" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A104">
         <v>103</v>
       </c>
@@ -5706,11 +5292,8 @@
       <c r="O104" t="s">
         <v>118</v>
       </c>
-      <c r="P104">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="105" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="105" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A105">
         <v>104</v>
       </c>
@@ -5747,11 +5330,8 @@
       <c r="O105" t="s">
         <v>118</v>
       </c>
-      <c r="P105">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="106" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="106" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A106">
         <v>105</v>
       </c>
@@ -5788,11 +5368,8 @@
       <c r="O106" t="s">
         <v>118</v>
       </c>
-      <c r="P106">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="107" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="107" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A107">
         <v>106</v>
       </c>
@@ -5829,11 +5406,8 @@
       <c r="O107" t="s">
         <v>119</v>
       </c>
-      <c r="P107">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="108" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="108" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A108">
         <v>107</v>
       </c>
@@ -5870,11 +5444,8 @@
       <c r="O108" t="s">
         <v>119</v>
       </c>
-      <c r="P108">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="109" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="109" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A109">
         <v>108</v>
       </c>
@@ -5911,11 +5482,8 @@
       <c r="O109" t="s">
         <v>119</v>
       </c>
-      <c r="P109">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="110" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="110" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A110">
         <v>109</v>
       </c>
@@ -5952,11 +5520,8 @@
       <c r="O110" t="s">
         <v>122</v>
       </c>
-      <c r="P110">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="111" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="111" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A111">
         <v>110</v>
       </c>
@@ -5993,11 +5558,8 @@
       <c r="O111" t="s">
         <v>125</v>
       </c>
-      <c r="P111">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="112" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="112" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A112">
         <v>111</v>
       </c>
@@ -6034,11 +5596,8 @@
       <c r="O112" t="s">
         <v>128</v>
       </c>
-      <c r="P112">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="113" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="113" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A113">
         <v>112</v>
       </c>
@@ -6075,11 +5634,8 @@
       <c r="O113" t="s">
         <v>131</v>
       </c>
-      <c r="P113">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="114" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="114" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A114">
         <v>113</v>
       </c>
@@ -6116,11 +5672,8 @@
       <c r="O114" t="s">
         <v>131</v>
       </c>
-      <c r="P114">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="115" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="115" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A115">
         <v>114</v>
       </c>
@@ -6157,11 +5710,8 @@
       <c r="O115" t="s">
         <v>134</v>
       </c>
-      <c r="P115">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="116" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="116" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A116">
         <v>115</v>
       </c>
@@ -6198,11 +5748,8 @@
       <c r="O116" t="s">
         <v>137</v>
       </c>
-      <c r="P116">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="117" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="117" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A117">
         <v>116</v>
       </c>
@@ -6239,11 +5786,8 @@
       <c r="O117" t="s">
         <v>137</v>
       </c>
-      <c r="P117">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="118" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="118" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A118">
         <v>117</v>
       </c>
@@ -6280,11 +5824,8 @@
       <c r="O118" t="s">
         <v>137</v>
       </c>
-      <c r="P118">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="119" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="119" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A119">
         <v>118</v>
       </c>
@@ -6321,11 +5862,8 @@
       <c r="O119" t="s">
         <v>140</v>
       </c>
-      <c r="P119">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="120" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="120" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A120">
         <v>119</v>
       </c>
@@ -6362,11 +5900,8 @@
       <c r="O120" t="s">
         <v>141</v>
       </c>
-      <c r="P120">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="121" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="121" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A121">
         <v>120</v>
       </c>
@@ -6403,11 +5938,8 @@
       <c r="O121" t="s">
         <v>141</v>
       </c>
-      <c r="P121">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="122" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="122" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A122">
         <v>121</v>
       </c>
@@ -6444,11 +5976,8 @@
       <c r="O122" t="s">
         <v>141</v>
       </c>
-      <c r="P122">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="123" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="123" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A123">
         <v>122</v>
       </c>
@@ -6485,11 +6014,8 @@
       <c r="O123" t="s">
         <v>141</v>
       </c>
-      <c r="P123">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="124" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="124" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A124">
         <v>123</v>
       </c>
@@ -6526,11 +6052,8 @@
       <c r="O124" t="s">
         <v>141</v>
       </c>
-      <c r="P124">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="125" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="125" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A125">
         <v>124</v>
       </c>
@@ -6567,14 +6090,8 @@
       <c r="O125" t="s">
         <v>141</v>
       </c>
-      <c r="P125">
-        <v>3</v>
-      </c>
-      <c r="Q125" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="126" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="126" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A126">
         <v>125</v>
       </c>
@@ -6611,11 +6128,8 @@
       <c r="O126" t="s">
         <v>144</v>
       </c>
-      <c r="P126">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="127" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="127" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A127">
         <v>126</v>
       </c>
@@ -6652,14 +6166,8 @@
       <c r="O127" t="s">
         <v>147</v>
       </c>
-      <c r="P127">
-        <v>3</v>
-      </c>
-      <c r="Q127" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="128" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="128" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A128">
         <v>127</v>
       </c>
@@ -6696,11 +6204,8 @@
       <c r="O128" t="s">
         <v>147</v>
       </c>
-      <c r="P128">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="129" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="129" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A129">
         <v>128</v>
       </c>
@@ -6737,11 +6242,8 @@
       <c r="O129" t="s">
         <v>147</v>
       </c>
-      <c r="P129">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="130" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="130" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A130">
         <v>129</v>
       </c>
@@ -6778,11 +6280,8 @@
       <c r="O130" t="s">
         <v>147</v>
       </c>
-      <c r="P130">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="131" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="131" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A131">
         <v>130</v>
       </c>
@@ -6819,11 +6318,8 @@
       <c r="O131" t="s">
         <v>150</v>
       </c>
-      <c r="P131">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="132" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="132" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A132">
         <v>131</v>
       </c>
@@ -6860,14 +6356,8 @@
       <c r="O132" t="s">
         <v>153</v>
       </c>
-      <c r="P132">
-        <v>3</v>
-      </c>
-      <c r="Q132" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="133" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="133" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A133">
         <v>132</v>
       </c>
@@ -6904,11 +6394,8 @@
       <c r="O133" t="s">
         <v>154</v>
       </c>
-      <c r="P133">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="134" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="134" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A134">
         <v>133</v>
       </c>
@@ -6945,11 +6432,8 @@
       <c r="O134" t="s">
         <v>154</v>
       </c>
-      <c r="P134">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="135" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="135" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A135">
         <v>134</v>
       </c>
@@ -6986,11 +6470,8 @@
       <c r="O135" t="s">
         <v>154</v>
       </c>
-      <c r="P135">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="136" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="136" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A136">
         <v>135</v>
       </c>
@@ -7027,11 +6508,8 @@
       <c r="O136" t="s">
         <v>157</v>
       </c>
-      <c r="P136">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="137" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="137" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A137">
         <v>136</v>
       </c>
@@ -7068,11 +6546,8 @@
       <c r="O137" t="s">
         <v>160</v>
       </c>
-      <c r="P137">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="138" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="138" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A138">
         <v>137</v>
       </c>
@@ -7109,11 +6584,8 @@
       <c r="O138" t="s">
         <v>160</v>
       </c>
-      <c r="P138">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="139" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="139" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A139">
         <v>138</v>
       </c>
@@ -7150,11 +6622,8 @@
       <c r="O139" t="s">
         <v>160</v>
       </c>
-      <c r="P139">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="140" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="140" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A140">
         <v>139</v>
       </c>
@@ -7191,11 +6660,8 @@
       <c r="O140" t="s">
         <v>160</v>
       </c>
-      <c r="P140">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="141" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="141" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A141">
         <v>140</v>
       </c>
@@ -7232,11 +6698,8 @@
       <c r="O141" t="s">
         <v>160</v>
       </c>
-      <c r="P141">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="142" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="142" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A142">
         <v>141</v>
       </c>
@@ -7273,11 +6736,8 @@
       <c r="O142" t="s">
         <v>160</v>
       </c>
-      <c r="P142">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="143" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="143" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A143">
         <v>142</v>
       </c>
@@ -7314,11 +6774,8 @@
       <c r="O143" t="s">
         <v>160</v>
       </c>
-      <c r="P143">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="144" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="144" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A144">
         <v>143</v>
       </c>
@@ -7355,11 +6812,8 @@
       <c r="O144" t="s">
         <v>161</v>
       </c>
-      <c r="P144">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="145" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="145" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A145">
         <v>144</v>
       </c>
@@ -7396,11 +6850,8 @@
       <c r="O145" t="s">
         <v>162</v>
       </c>
-      <c r="P145">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="146" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="146" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A146">
         <v>145</v>
       </c>
@@ -7437,11 +6888,8 @@
       <c r="O146" t="s">
         <v>163</v>
       </c>
-      <c r="P146">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="147" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="147" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A147">
         <v>146</v>
       </c>
@@ -7478,11 +6926,8 @@
       <c r="O147" t="s">
         <v>166</v>
       </c>
-      <c r="P147">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="148" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="148" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A148">
         <v>147</v>
       </c>
@@ -7519,11 +6964,8 @@
       <c r="O148" t="s">
         <v>166</v>
       </c>
-      <c r="P148">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="149" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="149" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A149">
         <v>148</v>
       </c>
@@ -7560,11 +7002,8 @@
       <c r="O149" t="s">
         <v>167</v>
       </c>
-      <c r="P149">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="150" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="150" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A150">
         <v>149</v>
       </c>
@@ -7601,14 +7040,8 @@
       <c r="O150" t="s">
         <v>170</v>
       </c>
-      <c r="P150">
-        <v>2</v>
-      </c>
-      <c r="Q150" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="151" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="151" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A151">
         <v>150</v>
       </c>
@@ -7645,11 +7078,8 @@
       <c r="O151" t="s">
         <v>173</v>
       </c>
-      <c r="P151">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="152" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="152" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A152">
         <v>151</v>
       </c>
@@ -7686,11 +7116,8 @@
       <c r="O152" t="s">
         <v>173</v>
       </c>
-      <c r="P152">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="153" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="153" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A153">
         <v>152</v>
       </c>
@@ -7727,11 +7154,8 @@
       <c r="O153" t="s">
         <v>173</v>
       </c>
-      <c r="P153">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="154" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="154" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A154">
         <v>153</v>
       </c>
@@ -7768,11 +7192,8 @@
       <c r="O154" t="s">
         <v>174</v>
       </c>
-      <c r="P154">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="155" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="155" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A155">
         <v>154</v>
       </c>
@@ -7809,11 +7230,8 @@
       <c r="O155" t="s">
         <v>176</v>
       </c>
-      <c r="P155">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="156" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="156" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A156">
         <v>155</v>
       </c>
@@ -7850,11 +7268,8 @@
       <c r="O156" t="s">
         <v>176</v>
       </c>
-      <c r="P156">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="157" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="157" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A157">
         <v>156</v>
       </c>
@@ -7891,11 +7306,8 @@
       <c r="O157" t="s">
         <v>176</v>
       </c>
-      <c r="P157">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="158" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="158" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A158">
         <v>157</v>
       </c>
@@ -7932,11 +7344,8 @@
       <c r="O158" t="s">
         <v>176</v>
       </c>
-      <c r="P158">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="159" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="159" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A159">
         <v>158</v>
       </c>
@@ -7973,11 +7382,8 @@
       <c r="O159" t="s">
         <v>176</v>
       </c>
-      <c r="P159">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="160" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="160" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A160">
         <v>159</v>
       </c>
@@ -8014,11 +7420,8 @@
       <c r="O160" t="s">
         <v>176</v>
       </c>
-      <c r="P160">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="161" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="161" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A161">
         <v>160</v>
       </c>
@@ -8055,11 +7458,8 @@
       <c r="O161" t="s">
         <v>176</v>
       </c>
-      <c r="P161">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="162" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="162" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A162">
         <v>161</v>
       </c>
@@ -8096,11 +7496,8 @@
       <c r="O162" t="s">
         <v>176</v>
       </c>
-      <c r="P162">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="163" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="163" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A163">
         <v>162</v>
       </c>
@@ -8137,11 +7534,8 @@
       <c r="O163" t="s">
         <v>176</v>
       </c>
-      <c r="P163">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="164" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="164" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A164">
         <v>163</v>
       </c>
@@ -8178,11 +7572,8 @@
       <c r="O164" t="s">
         <v>176</v>
       </c>
-      <c r="P164">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="165" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="165" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A165">
         <v>164</v>
       </c>
@@ -8219,11 +7610,8 @@
       <c r="O165" t="s">
         <v>176</v>
       </c>
-      <c r="P165">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="166" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="166" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A166">
         <v>165</v>
       </c>
@@ -8260,11 +7648,8 @@
       <c r="O166" t="s">
         <v>176</v>
       </c>
-      <c r="P166">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="167" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="167" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A167">
         <v>166</v>
       </c>
@@ -8301,11 +7686,8 @@
       <c r="O167" t="s">
         <v>176</v>
       </c>
-      <c r="P167">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="168" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="168" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A168">
         <v>167</v>
       </c>
@@ -8342,11 +7724,8 @@
       <c r="O168" t="s">
         <v>176</v>
       </c>
-      <c r="P168">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="169" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="169" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A169">
         <v>168</v>
       </c>
@@ -8383,11 +7762,8 @@
       <c r="O169" t="s">
         <v>176</v>
       </c>
-      <c r="P169">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="170" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="170" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A170">
         <v>169</v>
       </c>
@@ -8424,11 +7800,8 @@
       <c r="O170" t="s">
         <v>176</v>
       </c>
-      <c r="P170">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="171" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="171" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A171">
         <v>170</v>
       </c>
@@ -8471,11 +7844,8 @@
       <c r="O171" t="s">
         <v>179</v>
       </c>
-      <c r="Q171" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="172" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="172" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A172">
         <v>171</v>
       </c>
@@ -8518,11 +7888,8 @@
       <c r="O172" t="s">
         <v>179</v>
       </c>
-      <c r="P172">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="173" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="173" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A173">
         <v>172</v>
       </c>
@@ -8565,11 +7932,8 @@
       <c r="O173" t="s">
         <v>179</v>
       </c>
-      <c r="Q173" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="174" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="174" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A174">
         <v>173</v>
       </c>
@@ -8606,11 +7970,8 @@
       <c r="O174" t="s">
         <v>182</v>
       </c>
-      <c r="P174">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="175" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="175" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A175">
         <v>174</v>
       </c>
@@ -8647,11 +8008,8 @@
       <c r="O175" t="s">
         <v>182</v>
       </c>
-      <c r="P175">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="176" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="176" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A176">
         <v>175</v>
       </c>
@@ -8688,11 +8046,8 @@
       <c r="O176" t="s">
         <v>182</v>
       </c>
-      <c r="P176">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="177" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="177" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A177">
         <v>176</v>
       </c>
@@ -8729,11 +8084,8 @@
       <c r="O177" t="s">
         <v>182</v>
       </c>
-      <c r="P177">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="178" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="178" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A178">
         <v>177</v>
       </c>
@@ -8776,11 +8128,8 @@
       <c r="O178" t="s">
         <v>183</v>
       </c>
-      <c r="P178">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="179" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="179" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A179">
         <v>178</v>
       </c>
@@ -8823,11 +8172,8 @@
       <c r="O179" t="s">
         <v>186</v>
       </c>
-      <c r="P179">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="180" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="180" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A180">
         <v>179</v>
       </c>
@@ -8870,11 +8216,8 @@
       <c r="O180" t="s">
         <v>186</v>
       </c>
-      <c r="P180">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="181" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="181" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A181">
         <v>180</v>
       </c>
@@ -8917,11 +8260,8 @@
       <c r="O181" t="s">
         <v>186</v>
       </c>
-      <c r="P181">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="182" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="182" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A182">
         <v>181</v>
       </c>
@@ -8964,11 +8304,8 @@
       <c r="O182" t="s">
         <v>186</v>
       </c>
-      <c r="P182">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="183" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="183" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A183">
         <v>182</v>
       </c>
@@ -9005,11 +8342,8 @@
       <c r="O183" t="s">
         <v>187</v>
       </c>
-      <c r="P183">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="184" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="184" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A184">
         <v>183</v>
       </c>
@@ -9046,11 +8380,8 @@
       <c r="O184" t="s">
         <v>187</v>
       </c>
-      <c r="P184">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="185" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="185" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A185">
         <v>184</v>
       </c>
@@ -9087,11 +8418,8 @@
       <c r="O185" t="s">
         <v>187</v>
       </c>
-      <c r="P185">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="186" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="186" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A186">
         <v>185</v>
       </c>
@@ -9128,11 +8456,8 @@
       <c r="O186" t="s">
         <v>190</v>
       </c>
-      <c r="P186">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="187" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="187" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A187">
         <v>186</v>
       </c>
@@ -9169,11 +8494,8 @@
       <c r="O187" t="s">
         <v>193</v>
       </c>
-      <c r="P187">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="188" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="188" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A188">
         <v>187</v>
       </c>
@@ -9210,11 +8532,8 @@
       <c r="O188" t="s">
         <v>196</v>
       </c>
-      <c r="P188">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="189" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="189" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A189">
         <v>188</v>
       </c>
@@ -9251,11 +8570,8 @@
       <c r="O189" t="s">
         <v>199</v>
       </c>
-      <c r="P189">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="190" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="190" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A190">
         <v>189</v>
       </c>
@@ -9292,11 +8608,8 @@
       <c r="O190" t="s">
         <v>202</v>
       </c>
-      <c r="P190">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="191" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="191" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A191">
         <v>190</v>
       </c>
@@ -9339,11 +8652,8 @@
       <c r="O191" t="s">
         <v>203</v>
       </c>
-      <c r="P191">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="192" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="192" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A192">
         <v>191</v>
       </c>
@@ -9386,11 +8696,8 @@
       <c r="O192" t="s">
         <v>203</v>
       </c>
-      <c r="P192">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="193" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="193" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A193">
         <v>192</v>
       </c>
@@ -9433,11 +8740,8 @@
       <c r="O193" t="s">
         <v>203</v>
       </c>
-      <c r="P193">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="194" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="194" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A194">
         <v>193</v>
       </c>
@@ -9480,11 +8784,8 @@
       <c r="O194" t="s">
         <v>203</v>
       </c>
-      <c r="P194">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="195" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="195" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A195">
         <v>194</v>
       </c>
@@ -9527,11 +8828,8 @@
       <c r="O195" t="s">
         <v>203</v>
       </c>
-      <c r="P195">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="196" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="196" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A196">
         <v>195</v>
       </c>
@@ -9568,11 +8866,8 @@
       <c r="O196" t="s">
         <v>204</v>
       </c>
-      <c r="P196">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="197" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="197" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A197">
         <v>196</v>
       </c>
@@ -9609,11 +8904,8 @@
       <c r="O197" t="s">
         <v>207</v>
       </c>
-      <c r="P197">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="198" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="198" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A198">
         <v>197</v>
       </c>
@@ -9650,11 +8942,8 @@
       <c r="O198" t="s">
         <v>207</v>
       </c>
-      <c r="P198">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="199" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="199" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A199">
         <v>198</v>
       </c>
@@ -9691,11 +8980,8 @@
       <c r="O199" t="s">
         <v>207</v>
       </c>
-      <c r="P199">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="200" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="200" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A200">
         <v>199</v>
       </c>
@@ -9732,11 +9018,8 @@
       <c r="O200" t="s">
         <v>207</v>
       </c>
-      <c r="P200">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="201" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="201" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A201">
         <v>200</v>
       </c>
@@ -9773,11 +9056,8 @@
       <c r="O201" t="s">
         <v>207</v>
       </c>
-      <c r="P201">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="202" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="202" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A202">
         <v>201</v>
       </c>
@@ -9814,11 +9094,8 @@
       <c r="O202" t="s">
         <v>207</v>
       </c>
-      <c r="P202">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="203" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="203" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A203">
         <v>202</v>
       </c>
@@ -9855,11 +9132,8 @@
       <c r="O203" t="s">
         <v>207</v>
       </c>
-      <c r="P203">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="204" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="204" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A204">
         <v>203</v>
       </c>
@@ -9896,11 +9170,8 @@
       <c r="O204" t="s">
         <v>207</v>
       </c>
-      <c r="P204">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="205" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="205" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A205">
         <v>204</v>
       </c>
@@ -9937,11 +9208,8 @@
       <c r="O205" t="s">
         <v>208</v>
       </c>
-      <c r="P205">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="206" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="206" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A206">
         <v>205</v>
       </c>
@@ -9978,11 +9246,8 @@
       <c r="O206" t="s">
         <v>208</v>
       </c>
-      <c r="P206">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="207" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="207" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A207">
         <v>206</v>
       </c>
@@ -10019,11 +9284,8 @@
       <c r="O207" t="s">
         <v>211</v>
       </c>
-      <c r="P207">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="208" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="208" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A208">
         <v>207</v>
       </c>
@@ -10060,11 +9322,8 @@
       <c r="O208" t="s">
         <v>211</v>
       </c>
-      <c r="P208">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="209" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="209" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A209">
         <v>208</v>
       </c>
@@ -10101,11 +9360,8 @@
       <c r="O209" t="s">
         <v>211</v>
       </c>
-      <c r="P209">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="210" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="210" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A210">
         <v>209</v>
       </c>
@@ -10142,11 +9398,8 @@
       <c r="O210" t="s">
         <v>211</v>
       </c>
-      <c r="P210">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="211" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="211" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A211">
         <v>210</v>
       </c>
@@ -10183,11 +9436,8 @@
       <c r="O211" t="s">
         <v>211</v>
       </c>
-      <c r="P211">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="212" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="212" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A212">
         <v>211</v>
       </c>
@@ -10224,11 +9474,8 @@
       <c r="O212" t="s">
         <v>211</v>
       </c>
-      <c r="P212">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="213" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="213" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A213">
         <v>212</v>
       </c>
@@ -10265,11 +9512,8 @@
       <c r="O213" t="s">
         <v>211</v>
       </c>
-      <c r="P213">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="214" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="214" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A214">
         <v>213</v>
       </c>
@@ -10306,11 +9550,8 @@
       <c r="O214" t="s">
         <v>211</v>
       </c>
-      <c r="P214">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="215" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="215" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A215">
         <v>214</v>
       </c>
@@ -10347,11 +9588,8 @@
       <c r="O215" t="s">
         <v>211</v>
       </c>
-      <c r="P215">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="216" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="216" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A216">
         <v>215</v>
       </c>
@@ -10388,11 +9626,8 @@
       <c r="O216" t="s">
         <v>212</v>
       </c>
-      <c r="P216">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="217" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="217" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A217">
         <v>216</v>
       </c>
@@ -10429,11 +9664,8 @@
       <c r="O217" t="s">
         <v>215</v>
       </c>
-      <c r="P217">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="218" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="218" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A218">
         <v>217</v>
       </c>
@@ -10470,11 +9702,8 @@
       <c r="O218" t="s">
         <v>215</v>
       </c>
-      <c r="P218">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="219" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="219" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A219">
         <v>218</v>
       </c>
@@ -10511,11 +9740,8 @@
       <c r="O219" t="s">
         <v>216</v>
       </c>
-      <c r="P219">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="220" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="220" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A220">
         <v>219</v>
       </c>
@@ -10552,11 +9778,8 @@
       <c r="O220" t="s">
         <v>217</v>
       </c>
-      <c r="P220">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="221" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="221" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A221">
         <v>220</v>
       </c>
@@ -10593,11 +9816,8 @@
       <c r="O221" t="s">
         <v>220</v>
       </c>
-      <c r="P221">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="222" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="222" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A222">
         <v>221</v>
       </c>
@@ -10634,11 +9854,8 @@
       <c r="O222" t="s">
         <v>223</v>
       </c>
-      <c r="P222">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="223" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="223" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A223">
         <v>222</v>
       </c>
@@ -10675,11 +9892,8 @@
       <c r="O223" t="s">
         <v>226</v>
       </c>
-      <c r="P223">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="224" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="224" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A224">
         <v>223</v>
       </c>
@@ -10716,11 +9930,8 @@
       <c r="O224" t="s">
         <v>229</v>
       </c>
-      <c r="P224">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="225" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="225" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A225">
         <v>224</v>
       </c>
@@ -10757,14 +9968,8 @@
       <c r="O225" t="s">
         <v>232</v>
       </c>
-      <c r="P225">
-        <v>3</v>
-      </c>
-      <c r="Q225" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="226" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="226" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A226">
         <v>225</v>
       </c>
@@ -10801,11 +10006,8 @@
       <c r="O226" t="s">
         <v>233</v>
       </c>
-      <c r="P226">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="227" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="227" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A227">
         <v>226</v>
       </c>
@@ -10842,11 +10044,8 @@
       <c r="O227" t="s">
         <v>233</v>
       </c>
-      <c r="P227">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="228" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="228" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A228">
         <v>227</v>
       </c>
@@ -10883,11 +10082,8 @@
       <c r="O228" t="s">
         <v>236</v>
       </c>
-      <c r="P228">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="229" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="229" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A229">
         <v>228</v>
       </c>
@@ -10924,11 +10120,8 @@
       <c r="O229" t="s">
         <v>236</v>
       </c>
-      <c r="P229">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="230" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="230" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A230">
         <v>229</v>
       </c>
@@ -10965,11 +10158,8 @@
       <c r="O230" t="s">
         <v>236</v>
       </c>
-      <c r="P230">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="231" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="231" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A231">
         <v>230</v>
       </c>
@@ -11006,11 +10196,8 @@
       <c r="O231" t="s">
         <v>236</v>
       </c>
-      <c r="P231">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="232" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="232" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A232">
         <v>231</v>
       </c>
@@ -11047,11 +10234,8 @@
       <c r="O232" t="s">
         <v>236</v>
       </c>
-      <c r="P232">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="233" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="233" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A233">
         <v>232</v>
       </c>
@@ -11088,11 +10272,8 @@
       <c r="O233" t="s">
         <v>236</v>
       </c>
-      <c r="P233">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="234" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="234" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A234">
         <v>233</v>
       </c>
@@ -11129,11 +10310,8 @@
       <c r="O234" t="s">
         <v>236</v>
       </c>
-      <c r="P234">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="235" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="235" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A235">
         <v>234</v>
       </c>
@@ -11170,11 +10348,8 @@
       <c r="O235" t="s">
         <v>236</v>
       </c>
-      <c r="P235">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="236" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="236" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A236">
         <v>235</v>
       </c>
@@ -11211,11 +10386,8 @@
       <c r="O236" t="s">
         <v>236</v>
       </c>
-      <c r="P236">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="237" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="237" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A237">
         <v>236</v>
       </c>
@@ -11252,11 +10424,8 @@
       <c r="O237" t="s">
         <v>236</v>
       </c>
-      <c r="P237">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="238" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="238" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A238">
         <v>237</v>
       </c>
@@ -11293,11 +10462,8 @@
       <c r="O238" t="s">
         <v>236</v>
       </c>
-      <c r="P238">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="239" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="239" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A239">
         <v>238</v>
       </c>
@@ -11334,11 +10500,8 @@
       <c r="O239" t="s">
         <v>236</v>
       </c>
-      <c r="P239">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="240" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="240" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A240">
         <v>239</v>
       </c>
@@ -11375,11 +10538,8 @@
       <c r="O240" t="s">
         <v>236</v>
       </c>
-      <c r="P240">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="241" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="241" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A241">
         <v>240</v>
       </c>
@@ -11416,11 +10576,8 @@
       <c r="O241" t="s">
         <v>236</v>
       </c>
-      <c r="P241">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="242" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="242" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A242">
         <v>241</v>
       </c>
@@ -11457,11 +10614,8 @@
       <c r="O242" t="s">
         <v>236</v>
       </c>
-      <c r="P242">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="243" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="243" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A243">
         <v>242</v>
       </c>
@@ -11498,11 +10652,8 @@
       <c r="O243" t="s">
         <v>236</v>
       </c>
-      <c r="P243">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="244" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="244" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A244">
         <v>243</v>
       </c>
@@ -11539,11 +10690,8 @@
       <c r="O244" t="s">
         <v>236</v>
       </c>
-      <c r="P244">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="245" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="245" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A245">
         <v>244</v>
       </c>
@@ -11580,14 +10728,8 @@
       <c r="O245" t="s">
         <v>236</v>
       </c>
-      <c r="P245">
-        <v>4</v>
-      </c>
-      <c r="Q245" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="246" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="246" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A246">
         <v>245</v>
       </c>
@@ -11624,11 +10766,8 @@
       <c r="O246" t="s">
         <v>236</v>
       </c>
-      <c r="P246">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="247" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="247" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A247">
         <v>246</v>
       </c>
@@ -11665,11 +10804,8 @@
       <c r="O247" t="s">
         <v>239</v>
       </c>
-      <c r="P247">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="248" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="248" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A248">
         <v>247</v>
       </c>
@@ -11706,11 +10842,8 @@
       <c r="O248" t="s">
         <v>239</v>
       </c>
-      <c r="P248">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="249" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="249" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A249">
         <v>248</v>
       </c>
@@ -11747,11 +10880,8 @@
       <c r="O249" t="s">
         <v>239</v>
       </c>
-      <c r="P249">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="250" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="250" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A250">
         <v>249</v>
       </c>
@@ -11788,11 +10918,8 @@
       <c r="O250" t="s">
         <v>239</v>
       </c>
-      <c r="P250">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="251" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="251" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A251">
         <v>250</v>
       </c>
@@ -11829,11 +10956,8 @@
       <c r="O251" t="s">
         <v>239</v>
       </c>
-      <c r="P251">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="252" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="252" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A252">
         <v>251</v>
       </c>
@@ -11870,11 +10994,8 @@
       <c r="O252" t="s">
         <v>239</v>
       </c>
-      <c r="P252">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="253" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="253" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A253">
         <v>252</v>
       </c>
@@ -11911,11 +11032,8 @@
       <c r="O253" t="s">
         <v>242</v>
       </c>
-      <c r="P253">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="254" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="254" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A254">
         <v>253</v>
       </c>
@@ -11952,11 +11070,8 @@
       <c r="O254" t="s">
         <v>245</v>
       </c>
-      <c r="P254">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="255" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="255" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A255">
         <v>254</v>
       </c>
@@ -11993,11 +11108,8 @@
       <c r="O255" t="s">
         <v>248</v>
       </c>
-      <c r="P255">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="256" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="256" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A256">
         <v>255</v>
       </c>
@@ -12034,11 +11146,8 @@
       <c r="O256" t="s">
         <v>248</v>
       </c>
-      <c r="P256">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="257" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="257" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A257">
         <v>256</v>
       </c>
@@ -12075,11 +11184,8 @@
       <c r="O257" t="s">
         <v>248</v>
       </c>
-      <c r="P257">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="258" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="258" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A258">
         <v>257</v>
       </c>
@@ -12116,11 +11222,8 @@
       <c r="O258" t="s">
         <v>251</v>
       </c>
-      <c r="P258">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="259" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="259" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A259">
         <v>258</v>
       </c>
@@ -12157,11 +11260,8 @@
       <c r="O259" t="s">
         <v>254</v>
       </c>
-      <c r="P259">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="260" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="260" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A260">
         <v>259</v>
       </c>
@@ -12198,11 +11298,8 @@
       <c r="O260" t="s">
         <v>257</v>
       </c>
-      <c r="P260">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="261" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="261" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A261">
         <v>260</v>
       </c>
@@ -12239,14 +11336,8 @@
       <c r="O261" t="s">
         <v>260</v>
       </c>
-      <c r="P261">
-        <v>3</v>
-      </c>
-      <c r="Q261" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="262" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="262" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A262">
         <v>261</v>
       </c>
@@ -12283,11 +11374,8 @@
       <c r="O262" t="s">
         <v>260</v>
       </c>
-      <c r="P262">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="263" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="263" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A263">
         <v>262</v>
       </c>
@@ -12324,11 +11412,8 @@
       <c r="O263" t="s">
         <v>260</v>
       </c>
-      <c r="P263">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="264" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="264" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A264">
         <v>263</v>
       </c>
@@ -12365,11 +11450,8 @@
       <c r="O264" t="s">
         <v>263</v>
       </c>
-      <c r="P264">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="265" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="265" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A265">
         <v>264</v>
       </c>
@@ -12406,11 +11488,8 @@
       <c r="O265" t="s">
         <v>264</v>
       </c>
-      <c r="P265">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="266" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="266" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A266">
         <v>265</v>
       </c>
@@ -12447,11 +11526,8 @@
       <c r="O266" t="s">
         <v>264</v>
       </c>
-      <c r="P266">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="267" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="267" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A267">
         <v>266</v>
       </c>
@@ -12488,11 +11564,8 @@
       <c r="O267" t="s">
         <v>265</v>
       </c>
-      <c r="P267">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="268" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="268" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A268">
         <v>267</v>
       </c>
@@ -12529,11 +11602,8 @@
       <c r="O268" t="s">
         <v>266</v>
       </c>
-      <c r="P268">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="269" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="269" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A269">
         <v>268</v>
       </c>
@@ -12570,11 +11640,8 @@
       <c r="O269" t="s">
         <v>266</v>
       </c>
-      <c r="P269">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="270" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="270" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A270">
         <v>269</v>
       </c>
@@ -12611,11 +11678,8 @@
       <c r="O270" t="s">
         <v>266</v>
       </c>
-      <c r="P270">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="271" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="271" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A271">
         <v>270</v>
       </c>
@@ -12652,11 +11716,8 @@
       <c r="O271" t="s">
         <v>266</v>
       </c>
-      <c r="P271">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="272" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="272" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A272">
         <v>271</v>
       </c>
@@ -12693,11 +11754,8 @@
       <c r="O272" t="s">
         <v>267</v>
       </c>
-      <c r="P272">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="273" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="273" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A273">
         <v>272</v>
       </c>
@@ -12734,11 +11792,8 @@
       <c r="O273" t="s">
         <v>268</v>
       </c>
-      <c r="P273">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="274" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="274" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A274">
         <v>273</v>
       </c>
@@ -12775,11 +11830,8 @@
       <c r="O274" t="s">
         <v>269</v>
       </c>
-      <c r="P274">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="275" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="275" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A275">
         <v>274</v>
       </c>
@@ -12816,11 +11868,8 @@
       <c r="O275" t="s">
         <v>269</v>
       </c>
-      <c r="P275">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="276" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="276" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A276">
         <v>275</v>
       </c>
@@ -12857,11 +11906,8 @@
       <c r="O276" t="s">
         <v>269</v>
       </c>
-      <c r="P276">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="277" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="277" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A277">
         <v>276</v>
       </c>
@@ -12898,11 +11944,8 @@
       <c r="O277" t="s">
         <v>269</v>
       </c>
-      <c r="P277">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="278" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="278" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A278">
         <v>277</v>
       </c>
@@ -12939,11 +11982,8 @@
       <c r="O278" t="s">
         <v>272</v>
       </c>
-      <c r="P278">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="279" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="279" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A279">
         <v>278</v>
       </c>
@@ -12980,11 +12020,8 @@
       <c r="O279" t="s">
         <v>272</v>
       </c>
-      <c r="P279">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="280" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="280" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A280">
         <v>279</v>
       </c>
@@ -13021,11 +12058,8 @@
       <c r="O280" t="s">
         <v>272</v>
       </c>
-      <c r="P280">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="281" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="281" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A281">
         <v>280</v>
       </c>
@@ -13062,11 +12096,8 @@
       <c r="O281" t="s">
         <v>272</v>
       </c>
-      <c r="P281">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="282" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="282" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A282">
         <v>281</v>
       </c>
@@ -13103,11 +12134,8 @@
       <c r="O282" t="s">
         <v>272</v>
       </c>
-      <c r="P282">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="283" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="283" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A283">
         <v>282</v>
       </c>
@@ -13144,11 +12172,8 @@
       <c r="O283" t="s">
         <v>272</v>
       </c>
-      <c r="P283">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="284" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="284" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A284">
         <v>283</v>
       </c>
@@ -13185,11 +12210,8 @@
       <c r="O284" t="s">
         <v>273</v>
       </c>
-      <c r="P284">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="285" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="285" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A285">
         <v>284</v>
       </c>
@@ -13226,11 +12248,8 @@
       <c r="O285" t="s">
         <v>273</v>
       </c>
-      <c r="P285">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="286" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="286" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A286">
         <v>285</v>
       </c>
@@ -13267,11 +12286,8 @@
       <c r="O286" t="s">
         <v>276</v>
       </c>
-      <c r="P286">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="287" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="287" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A287">
         <v>286</v>
       </c>
@@ -13308,11 +12324,8 @@
       <c r="O287" t="s">
         <v>276</v>
       </c>
-      <c r="P287">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="288" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="288" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A288">
         <v>287</v>
       </c>
@@ -13349,11 +12362,8 @@
       <c r="O288" t="s">
         <v>276</v>
       </c>
-      <c r="P288">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="289" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="289" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A289">
         <v>288</v>
       </c>
@@ -13390,11 +12400,8 @@
       <c r="O289" t="s">
         <v>276</v>
       </c>
-      <c r="P289">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="290" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="290" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A290">
         <v>289</v>
       </c>
@@ -13431,11 +12438,8 @@
       <c r="O290" t="s">
         <v>276</v>
       </c>
-      <c r="P290">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="291" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="291" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A291">
         <v>290</v>
       </c>
@@ -13472,11 +12476,8 @@
       <c r="O291" t="s">
         <v>279</v>
       </c>
-      <c r="P291">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="292" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="292" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A292">
         <v>291</v>
       </c>
@@ -13513,14 +12514,8 @@
       <c r="O292" t="s">
         <v>280</v>
       </c>
-      <c r="P292">
-        <v>1</v>
-      </c>
-      <c r="Q292" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="293" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="293" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A293">
         <v>292</v>
       </c>
@@ -13557,11 +12552,8 @@
       <c r="O293" t="s">
         <v>280</v>
       </c>
-      <c r="P293">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="294" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="294" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A294">
         <v>293</v>
       </c>
@@ -13598,11 +12590,8 @@
       <c r="O294" t="s">
         <v>280</v>
       </c>
-      <c r="P294">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="295" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="295" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A295">
         <v>294</v>
       </c>
@@ -13639,11 +12628,8 @@
       <c r="O295" t="s">
         <v>280</v>
       </c>
-      <c r="P295">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="296" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="296" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A296">
         <v>295</v>
       </c>
@@ -13680,11 +12666,8 @@
       <c r="O296" t="s">
         <v>280</v>
       </c>
-      <c r="P296">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="297" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="297" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A297">
         <v>296</v>
       </c>
@@ -13721,11 +12704,8 @@
       <c r="O297" t="s">
         <v>280</v>
       </c>
-      <c r="P297">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="298" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="298" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A298">
         <v>297</v>
       </c>
@@ -13762,11 +12742,8 @@
       <c r="O298" t="s">
         <v>280</v>
       </c>
-      <c r="P298">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="299" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="299" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A299">
         <v>298</v>
       </c>
@@ -13803,11 +12780,8 @@
       <c r="O299" t="s">
         <v>281</v>
       </c>
-      <c r="P299">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="300" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="300" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A300">
         <v>299</v>
       </c>
@@ -13844,11 +12818,8 @@
       <c r="O300" t="s">
         <v>284</v>
       </c>
-      <c r="P300">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="301" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="301" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A301">
         <v>300</v>
       </c>
@@ -13885,11 +12856,8 @@
       <c r="O301" t="s">
         <v>285</v>
       </c>
-      <c r="P301">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="302" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="302" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A302">
         <v>301</v>
       </c>
@@ -13926,11 +12894,8 @@
       <c r="O302" t="s">
         <v>285</v>
       </c>
-      <c r="P302">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="303" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="303" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A303">
         <v>302</v>
       </c>
@@ -13967,11 +12932,8 @@
       <c r="O303" t="s">
         <v>288</v>
       </c>
-      <c r="P303">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="304" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="304" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A304">
         <v>303</v>
       </c>
@@ -14008,14 +12970,8 @@
       <c r="O304" t="s">
         <v>288</v>
       </c>
-      <c r="P304">
-        <v>3</v>
-      </c>
-      <c r="Q304" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="305" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="305" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A305">
         <v>304</v>
       </c>
@@ -14052,11 +13008,8 @@
       <c r="O305" t="s">
         <v>288</v>
       </c>
-      <c r="P305">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="306" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="306" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A306">
         <v>305</v>
       </c>
@@ -14093,11 +13046,8 @@
       <c r="O306" t="s">
         <v>288</v>
       </c>
-      <c r="Q306" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="307" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="307" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A307">
         <v>306</v>
       </c>
@@ -14134,11 +13084,8 @@
       <c r="O307" t="s">
         <v>291</v>
       </c>
-      <c r="P307">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="308" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="308" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A308">
         <v>307</v>
       </c>
@@ -14175,11 +13122,8 @@
       <c r="O308" t="s">
         <v>291</v>
       </c>
-      <c r="P308">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="309" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="309" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A309">
         <v>308</v>
       </c>
@@ -14216,14 +13160,8 @@
       <c r="O309" t="s">
         <v>294</v>
       </c>
-      <c r="P309">
-        <v>4</v>
-      </c>
-      <c r="Q309" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="310" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="310" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A310">
         <v>309</v>
       </c>
@@ -14260,11 +13198,8 @@
       <c r="O310" t="s">
         <v>294</v>
       </c>
-      <c r="P310">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="311" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="311" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A311">
         <v>310</v>
       </c>
@@ -14301,11 +13236,8 @@
       <c r="O311" t="s">
         <v>294</v>
       </c>
-      <c r="P311">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="312" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="312" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A312">
         <v>311</v>
       </c>
@@ -14342,11 +13274,8 @@
       <c r="O312" t="s">
         <v>294</v>
       </c>
-      <c r="P312">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="313" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="313" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A313">
         <v>312</v>
       </c>
@@ -14383,11 +13312,8 @@
       <c r="O313" t="s">
         <v>297</v>
       </c>
-      <c r="P313">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="314" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="314" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A314">
         <v>313</v>
       </c>
@@ -14424,11 +13350,8 @@
       <c r="O314" t="s">
         <v>298</v>
       </c>
-      <c r="P314">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="315" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="315" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A315">
         <v>314</v>
       </c>
@@ -14465,11 +13388,8 @@
       <c r="O315" t="s">
         <v>301</v>
       </c>
-      <c r="P315">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="316" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="316" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A316">
         <v>315</v>
       </c>
@@ -14506,11 +13426,8 @@
       <c r="O316" t="s">
         <v>301</v>
       </c>
-      <c r="P316">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="317" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="317" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A317">
         <v>316</v>
       </c>
@@ -14547,11 +13464,8 @@
       <c r="O317" t="s">
         <v>301</v>
       </c>
-      <c r="P317">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="318" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="318" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A318">
         <v>317</v>
       </c>
@@ -14588,11 +13502,8 @@
       <c r="O318" t="s">
         <v>301</v>
       </c>
-      <c r="P318">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="319" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="319" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A319">
         <v>318</v>
       </c>
@@ -14629,14 +13540,8 @@
       <c r="O319" t="s">
         <v>301</v>
       </c>
-      <c r="P319">
-        <v>2</v>
-      </c>
-      <c r="Q319" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="320" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="320" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A320">
         <v>319</v>
       </c>
@@ -14673,14 +13578,8 @@
       <c r="O320" t="s">
         <v>301</v>
       </c>
-      <c r="P320">
-        <v>2</v>
-      </c>
-      <c r="Q320" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="321" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="321" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A321">
         <v>320</v>
       </c>
@@ -14717,11 +13616,8 @@
       <c r="O321" t="s">
         <v>304</v>
       </c>
-      <c r="P321">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="322" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="322" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A322">
         <v>321</v>
       </c>
@@ -14758,15 +13654,8 @@
       <c r="O322" t="s">
         <v>307</v>
       </c>
-      <c r="P322">
-        <v>4</v>
-      </c>
-      <c r="Q322" t="s">
-        <v>313</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q322" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>